<commit_message>
partial process on tech model development and linkage, NOT TESTED
</commit_message>
<xml_diff>
--- a/src/technology/simple-electrolysis/simple-electrolysis.xlsx
+++ b/src/technology/simple-electrolysis/simple-electrolysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\simple-electrolysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561ABD9E-E498-4104-BDAC-1135E6BE9A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A7E057-6322-48FD-8743-E1861F26CA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30990" yWindow="345" windowWidth="17730" windowHeight="15120" xr2:uid="{021BDB00-52DC-4A4E-ACEA-9258FAE2C700}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="710" activeTab="7" xr2:uid="{021BDB00-52DC-4A4E-ACEA-9258FAE2C700}"/>
   </bookViews>
   <sheets>
     <sheet name="designs" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="parameters" sheetId="5" r:id="rId5"/>
     <sheet name="results" sheetId="6" r:id="rId6"/>
     <sheet name="tranches" sheetId="7" r:id="rId7"/>
+    <sheet name="metadata" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,8 +42,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={3B508C36-D070-4D26-B7F0-89DB78A615D1}</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{3B508C36-D070-4D26-B7F0-89DB78A615D1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Possibly FYI message for funding amounts that are very small, say 5% or less of maximum or less than 25% of the smallest tranche for a category</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="106">
   <si>
     <t>Technology</t>
   </si>
@@ -330,19 +349,62 @@
   </si>
   <si>
     <t>Amount</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Investment Amount</t>
+  </si>
+  <si>
+    <t>Maximum</t>
+  </si>
+  <si>
+    <t>Maximum funding amounts are decided during scenario development in collaboration with the decision-maker.</t>
+  </si>
+  <si>
+    <t>No Funding</t>
+  </si>
+  <si>
+    <t>Low Funding</t>
+  </si>
+  <si>
+    <t>Assigning low funding amounts may result in over-estimation of impacts. For best results, assign $tranche or more dollars.</t>
+  </si>
+  <si>
+    <t>Assigning no funding to a category corresponds to the current state of technology for parameters and variables affected by research in that category.</t>
+  </si>
+  <si>
+    <t>Benchtop scale electrolysis system that splits water into hydrogen and oxygen. For demonstration only.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -365,9 +427,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,10 +448,16 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Hanes, Rebecca" id="{918CADAA-C70D-420C-B384-C6E3C82AAAFE}" userId="Hanes, Rebecca" providerId="None"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -426,7 +495,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -532,7 +601,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -674,22 +743,30 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B5" dT="2025-06-23T15:15:49.89" personId="{918CADAA-C70D-420C-B384-C6E3C82AAAFE}" id="{3B508C36-D070-4D26-B7F0-89DB78A615D1}">
+    <text>Possibly FYI message for funding amounts that are very small, say 5% or less of maximum or less than 25% of the smallest tranche for a category</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{768C47FA-A48E-4158-95EE-1019738EA2E7}">
   <dimension ref="A1:G49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -712,7 +789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -732,7 +809,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -752,7 +829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -772,7 +849,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -792,7 +869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -812,7 +889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -832,7 +909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -855,7 +932,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -875,7 +952,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -895,7 +972,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -915,7 +992,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -935,7 +1012,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -955,7 +1032,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -975,7 +1052,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -995,7 +1072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -1015,7 +1092,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1035,7 +1112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -1055,7 +1132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -1075,7 +1152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -1098,7 +1175,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -1118,7 +1195,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -1138,7 +1215,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -1158,7 +1235,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>6</v>
       </c>
@@ -1178,7 +1255,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -1198,7 +1275,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>6</v>
       </c>
@@ -1218,7 +1295,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -1238,7 +1315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>6</v>
       </c>
@@ -1258,7 +1335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>6</v>
       </c>
@@ -1278,7 +1355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -1298,7 +1375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -1318,7 +1395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -1341,7 +1418,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -1361,7 +1438,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -1381,7 +1458,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -1401,7 +1478,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -1421,7 +1498,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -1441,7 +1518,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -1461,7 +1538,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -1481,7 +1558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -1501,7 +1578,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -1521,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>6</v>
       </c>
@@ -1541,7 +1618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>6</v>
       </c>
@@ -1561,7 +1638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -1584,7 +1661,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -1604,7 +1681,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -1624,7 +1701,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -1644,7 +1721,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -1664,7 +1741,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1692,9 +1769,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B06E9135-CC92-4566-BC27-870212F980DF}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1720,7 +1797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1751,9 +1828,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB279C25-BB03-4F81-BF04-3441E556B5A5}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1773,7 +1850,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1790,7 +1867,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1807,7 +1884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1824,7 +1901,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1841,7 +1918,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1858,7 +1935,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1875,7 +1952,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1892,7 +1969,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1917,15 +1994,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E8DDB52-2793-4513-A7DB-EE354AA78557}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>65</v>
       </c>
@@ -1939,7 +2016,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -1950,7 +2027,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -1961,7 +2038,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -1972,7 +2049,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>72</v>
       </c>
@@ -1991,9 +2068,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D60756-8727-469C-BF07-9640ADCA9D3D}">
   <dimension ref="A1:G41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2016,7 +2093,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2036,7 +2113,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2056,7 +2133,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2076,7 +2153,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2096,7 +2173,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2116,7 +2193,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2136,7 +2213,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -2156,7 +2233,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -2176,7 +2253,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -2199,7 +2276,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -2222,7 +2299,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -2242,7 +2319,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -2262,7 +2339,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -2282,7 +2359,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -2302,7 +2379,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -2322,7 +2399,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -2342,7 +2419,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -2362,7 +2439,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>6</v>
       </c>
@@ -2382,7 +2459,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>6</v>
       </c>
@@ -2405,7 +2482,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>6</v>
       </c>
@@ -2428,7 +2505,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>6</v>
       </c>
@@ -2448,7 +2525,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -2468,7 +2545,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>6</v>
       </c>
@@ -2488,7 +2565,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -2508,7 +2585,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>6</v>
       </c>
@@ -2528,7 +2605,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>6</v>
       </c>
@@ -2548,7 +2625,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>6</v>
       </c>
@@ -2568,7 +2645,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>6</v>
       </c>
@@ -2588,7 +2665,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>6</v>
       </c>
@@ -2611,7 +2688,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>6</v>
       </c>
@@ -2634,7 +2711,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>6</v>
       </c>
@@ -2654,7 +2731,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>6</v>
       </c>
@@ -2674,7 +2751,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2694,7 +2771,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -2714,7 +2791,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>6</v>
       </c>
@@ -2734,7 +2811,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>6</v>
       </c>
@@ -2754,7 +2831,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -2774,7 +2851,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -2794,7 +2871,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -2817,7 +2894,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -2848,9 +2925,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{760878E9-3E08-4F0E-93DC-70B8D93093AE}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2867,7 +2944,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2881,7 +2958,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2895,7 +2972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2909,7 +2986,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2923,7 +3000,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -2937,7 +3014,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -2959,13 +3036,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6483DD-2255-49BA-BAE9-23EDEC3285E4}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>66</v>
       </c>
@@ -2979,7 +3056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -2990,7 +3067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -3001,7 +3078,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -3012,7 +3089,7 @@
         <v>2500000</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>69</v>
       </c>
@@ -3026,4 +3103,112 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F37A774-2E57-4B0A-B004-15FA93317D42}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>